<commit_message>
Adding automatic mission segment state generation.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/Mission_Profile.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/Mission_Profile.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F93BE51-29E8-4F66-BAAE-F8B420BB9A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53A170FA-C87B-4C04-87E1-14D331796985}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" activeTab="1" xr2:uid="{5FD27DBB-5210-421F-BEEA-403866C08751}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="27">
   <si>
     <t>Startup</t>
   </si>
@@ -109,6 +109,15 @@
   </si>
   <si>
     <t>Time (min)</t>
+  </si>
+  <si>
+    <t>DryorWet</t>
+  </si>
+  <si>
+    <t>Dry</t>
+  </si>
+  <si>
+    <t>Wet</t>
   </si>
 </sst>
 </file>
@@ -351,14 +360,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <fill>
         <patternFill>
@@ -452,10 +454,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="0A0A0A"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FAFAFA"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -784,7 +786,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C3EDFB2-1219-4035-B524-6E37F4BFF669}">
-  <dimension ref="A4:N15"/>
+  <dimension ref="A4:N16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="16.85546875" customWidth="1"/>
@@ -1187,9 +1189,47 @@
         <v>0.91400000000000003</v>
       </c>
     </row>
+    <row r="16" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C16" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="L16" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="M16" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="N16" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="D6:N15">
+  <conditionalFormatting sqref="D6:N16">
     <cfRule type="containsBlanks" dxfId="0" priority="1">
       <formula>LEN(TRIM(D6))=0</formula>
     </cfRule>

</xml_diff>

<commit_message>
Added propulsion1. Moved "get_engine_type" to "PropulsionUtils."
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/Mission_Profile.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/Mission_Profile.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53A170FA-C87B-4C04-87E1-14D331796985}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9D41309-E2B1-48EA-8B79-51F15CF82826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" activeTab="1" xr2:uid="{5FD27DBB-5210-421F-BEEA-403866C08751}"/>
   </bookViews>
@@ -111,13 +111,13 @@
     <t>Time (min)</t>
   </si>
   <si>
-    <t>DryorWet</t>
-  </si>
-  <si>
     <t>Dry</t>
   </si>
   <si>
     <t>Wet</t>
+  </si>
+  <si>
+    <t>Dry or Wet</t>
   </si>
 </sst>
 </file>
@@ -1136,19 +1136,19 @@
         <v>2.7E-2</v>
       </c>
       <c r="J14" s="6">
-        <v>1.7000000000000001E-2</v>
+        <v>2.7E-2</v>
       </c>
       <c r="K14" s="6">
-        <v>1.7000000000000001E-2</v>
+        <v>2.7E-2</v>
       </c>
       <c r="L14" s="6">
-        <v>1.7000000000000001E-2</v>
+        <v>2.7E-2</v>
       </c>
       <c r="M14" s="6">
-        <v>1.7000000000000001E-2</v>
+        <v>2.7E-2</v>
       </c>
       <c r="N14" s="6">
-        <v>1.7000000000000001E-2</v>
+        <v>2.7E-2</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1191,40 +1191,40 @@
     </row>
     <row r="16" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C16" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="E16" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="I16" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="J16" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F16" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="I16" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="J16" s="5" t="s">
-        <v>26</v>
-      </c>
       <c r="K16" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L16" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="N16" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Modularized mission segment setup computations.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/Mission_Profile.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/Mission_Profile.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5456C962-E49E-494B-A44C-97BF8605C357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6522DA05-673C-4AA3-870C-54573F647B7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22668" yWindow="1488" windowWidth="21600" windowHeight="11508" activeTab="1" xr2:uid="{5FD27DBB-5210-421F-BEEA-403866C08751}"/>
+    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" activeTab="1" xr2:uid="{5FD27DBB-5210-421F-BEEA-403866C08751}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -108,13 +108,13 @@
     <t>Time (min)</t>
   </si>
   <si>
-    <t>Dry</t>
-  </si>
-  <si>
-    <t>Wet</t>
-  </si>
-  <si>
     <t>Dry or Wet</t>
+  </si>
+  <si>
+    <t>"Dry"</t>
+  </si>
+  <si>
+    <t>"Wet"</t>
   </si>
 </sst>
 </file>
@@ -451,10 +451,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="0A0A0A"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FAFAFA"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -1155,37 +1155,37 @@
     </row>
     <row r="16" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C16" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="I16" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D16" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I16" s="5" t="s">
+      <c r="J16" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="K16" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="J16" s="5" t="s">
+      <c r="L16" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="K16" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="L16" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="M16" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>